<commit_message>
Update Data sales.xlsx & Master produk.xlsx datasets
</commit_message>
<xml_diff>
--- a/Master produk.xlsx
+++ b/Master produk.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Argo\Project AI\DOI BULANAN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78196469-45CD-44F8-B3AB-A1B8D58F2C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BDEFC1-6247-4C2D-8683-051B46B302FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A4E4CA0-3C41-4699-9069-61742CAEF447}"/>
   </bookViews>
@@ -16875,8 +16875,8 @@
         <v>1278</v>
       </c>
       <c r="J300">
-        <f>368*587</f>
-        <v>216016</v>
+        <f>368</f>
+        <v>368</v>
       </c>
       <c r="K300" t="s">
         <v>1326</v>
@@ -16918,8 +16918,8 @@
         <v>1278</v>
       </c>
       <c r="J301">
-        <f>370*587</f>
-        <v>217190</v>
+        <f>370</f>
+        <v>370</v>
       </c>
       <c r="K301" t="s">
         <v>1326</v>

</xml_diff>